<commit_message>
Adding filters in MyAttendance
</commit_message>
<xml_diff>
--- a/attendance_template.xlsx
+++ b/attendance_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yussif\Full Stack Dev\Iken\EMS_IKEN_Intern\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5E8784-BE42-4463-886C-CBD5767982CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B8A9A8-2BC8-4907-B829-45CB913D23F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1104,7 +1104,7 @@
         <v>14</v>
       </c>
       <c r="C52" s="3">
-        <v>0.42708333333333331</v>
+        <v>0.4375</v>
       </c>
       <c r="D52" s="3">
         <v>0.75</v>

</xml_diff>